<commit_message>
Fix optical alignment and audit Dayova template layouts
</commit_message>
<xml_diff>
--- a/brand/templates/dist/Dayova-Workbook.xlsx
+++ b/brand/templates/dist/Dayova-Workbook.xlsx
@@ -168,33 +168,33 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -203,10 +203,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -236,7 +236,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>

<commit_message>
Add original Dayova logo to template cover and start pages
</commit_message>
<xml_diff>
--- a/brand/templates/dist/Dayova-Workbook.xlsx
+++ b/brand/templates/dist/Dayova-Workbook.xlsx
@@ -421,6 +421,36 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>8</col>
+      <colOff>800100</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="800100" cy="800100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>4</col>
       <colOff>0</colOff>
       <row>14</row>
@@ -2093,16 +2123,17 @@
       <c r="J110" s="1" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B2:J3"/>
     <mergeCell ref="B16:J17"/>
     <mergeCell ref="B19:J20"/>
     <mergeCell ref="B10:J11"/>
     <mergeCell ref="B6:J7"/>
+    <mergeCell ref="I2:J3"/>
     <mergeCell ref="B23:J25"/>
     <mergeCell ref="B9:J9"/>
     <mergeCell ref="B18:J18"/>
+    <mergeCell ref="B2:H3"/>
     <mergeCell ref="B4:J4"/>
     <mergeCell ref="B12:J12"/>
     <mergeCell ref="B13:J14"/>
@@ -2110,6 +2141,7 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>